<commit_message>
Actualizacao da leitura de graficos e qualidade de sessoes
</commit_message>
<xml_diff>
--- a/Qualidade_Sessoes.xlsx
+++ b/Qualidade_Sessoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -434,27 +434,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>28-Apr-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -464,22 +464,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -489,17 +489,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3918786000010071142</t>
+          <t>3918786000010125016</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -511,27 +511,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25-Apr-2026</t>
+          <t>21-Apr-2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -541,22 +541,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -566,49 +566,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3918786000010071140</t>
+          <t>3918786000010125014</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>14-Apr-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -618,22 +618,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -643,17 +643,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>30</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>3918786000010071138</t>
+          <t>3918786000010125012</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -665,27 +665,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>08-Apr-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -695,42 +695,42 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>26</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>3918786000010071136</t>
+          <t>3918786000010125010</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -742,22 +742,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>31-Mar-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -772,22 +772,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>26</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3918786000010071134</t>
+          <t>3918786000010125008</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -819,72 +819,72 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>24-Mar-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3918786000010015036</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>27</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>3918786000010071132</t>
+          <t>3918786000010125006</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -896,27 +896,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>17-Mar-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -926,22 +926,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3918786000010015034</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -951,17 +951,17 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>30</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>3918786000010071130</t>
+          <t>3918786000010125004</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -973,27 +973,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>10-Mar-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3918786000006032015</t>
+          <t>3918786000006032027</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mainote Momade</t>
+          <t>Agostinho Júlio Adelino</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3918786000010015034</t>
+          <t>3918786000010015014</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1028,17 +1028,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>30</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>3918786000010071128</t>
+          <t>3918786000010125002</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1080,22 +1080,22 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3918786000010015034</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>3918786000010071126</t>
+          <t>3918786000010071142</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18-Apr-2026</t>
+          <t>25-Apr-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1157,37 +1157,37 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3918786000010015038</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>25</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>3918786000010071124</t>
+          <t>3918786000010071140</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1234,22 +1234,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3918786000010015038</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>3918786000010071122</t>
+          <t>3918786000010071138</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1311,37 +1311,37 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3918786000010015038</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>3918786000010071120</t>
+          <t>3918786000010071136</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1388,37 +1388,37 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3918786000010015034</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>15</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>3918786000010071118</t>
+          <t>3918786000010071134</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1455,37 +1455,37 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3918786000010015034</t>
+          <t>3918786000010015036</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>JARDIM</t>
+          <t>MURROMONE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>3918786000010071116</t>
+          <t>3918786000010071132</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1557,22 +1557,22 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>3918786000010071114</t>
+          <t>3918786000010071130</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1589,75 +1589,691 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3918786000010015034</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Sessão_5</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>3918786000010071128</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>3918786000010015034</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Sessão_4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>3918786000010071126</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>3918786000010015038</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>3918786000010071124</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>3918786000010015038</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>3918786000010071122</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>3918786000010015038</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>3918786000010071120</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>3918786000010015034</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>3918786000010071118</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>3918786000010015034</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>3918786000010071116</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>18-Apr-2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3918786000006032015</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mainote Momade</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3918786000010015034</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>JARDIM</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>3918786000010071114</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>10-Mar-2026</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Marlene João Alfredo</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>3918786000006032043</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Marlene João Alfredo</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>NAMARIESSA</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>3918786000010015004</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>NAMARIESSA</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>3918786000010015294</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>Ribaue</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1666,4 +2282,271 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
+    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F32588A0-EB87-4A3C-B29A-8EC6DF0F2EEB}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E53F34B-A4DC-4293-A35A-78FDC71CDCCE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{254E9B65-A011-43F5-807A-8FAA662601D3}"/>
 </file>
</xml_diff>